<commit_message>
Oct 25, 2026, 12:56 PM
</commit_message>
<xml_diff>
--- a/La Liga 26-27.xlsx
+++ b/La Liga 26-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E44B3B5-F5C2-4A8C-A407-99AF18B1251E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9843AC58-8270-499D-AC7E-26A490D60E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="404" xr2:uid="{2BF33204-32E8-4B40-BC26-7C459B7DAA69}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="194">
   <si>
     <t>date</t>
   </si>
@@ -619,6 +619,9 @@
   <si>
     <t>Fri 23 October, 21:00</t>
   </si>
+  <si>
+    <t>Sun 18 October, 21:00</t>
+  </si>
 </sst>
 </file>
 
@@ -1043,7 +1046,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886C5DDF-1A39-4E94-A421-1D1D9FD99BEC}">
-  <dimension ref="A1:CK89"/>
+  <dimension ref="A1:CK90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -1373,7 +1376,7 @@
         <v>52</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H89" si="0">100-G2</f>
+        <f t="shared" ref="H2:H90" si="0">100-G2</f>
         <v>48</v>
       </c>
       <c r="I2">
@@ -24126,184 +24129,184 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="2:88" ht="30">
-      <c r="B88" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="C88" t="s">
-        <v>88</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>91</v>
+    <row r="88" spans="2:88" ht="25.5">
+      <c r="B88" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D88" t="s">
+        <v>90</v>
       </c>
       <c r="E88">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F88">
         <v>1</v>
       </c>
       <c r="G88">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="H88">
         <f t="shared" si="0"/>
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="I88">
-        <v>0.56999999999999995</v>
+        <v>2.2799999999999998</v>
       </c>
       <c r="J88">
-        <v>2.25</v>
+        <v>0.75</v>
       </c>
       <c r="K88">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="L88">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="M88">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N88">
         <v>5</v>
       </c>
       <c r="O88">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P88">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q88">
         <v>0</v>
       </c>
       <c r="R88">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S88">
-        <v>181</v>
+        <v>605</v>
       </c>
       <c r="T88">
-        <v>521</v>
+        <v>280</v>
       </c>
       <c r="U88">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="V88">
+        <v>14</v>
+      </c>
+      <c r="W88">
+        <v>1</v>
+      </c>
+      <c r="X88">
+        <v>2</v>
+      </c>
+      <c r="Y88" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z88" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA88">
+        <v>5</v>
+      </c>
+      <c r="AB88">
+        <v>4</v>
+      </c>
+      <c r="AC88">
+        <v>2</v>
+      </c>
+      <c r="AD88">
+        <v>2</v>
+      </c>
+      <c r="AE88">
+        <v>0</v>
+      </c>
+      <c r="AF88">
+        <v>0</v>
+      </c>
+      <c r="AG88">
+        <v>10</v>
+      </c>
+      <c r="AH88">
         <v>9</v>
       </c>
-      <c r="W88">
-        <v>8</v>
-      </c>
-      <c r="X88">
-        <v>8</v>
-      </c>
-      <c r="Y88" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z88" t="s">
-        <v>89</v>
-      </c>
-      <c r="AA88">
-        <v>4</v>
-      </c>
-      <c r="AB88">
-        <v>8</v>
-      </c>
-      <c r="AC88">
-        <v>4</v>
-      </c>
-      <c r="AD88">
-        <v>8</v>
-      </c>
-      <c r="AE88">
-        <v>1</v>
-      </c>
-      <c r="AF88">
-        <v>0</v>
-      </c>
-      <c r="AG88">
-        <v>4</v>
-      </c>
-      <c r="AH88">
-        <v>8</v>
-      </c>
       <c r="AI88">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AJ88">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="AK88">
-        <v>0.41</v>
+        <v>1.46</v>
       </c>
       <c r="AL88">
-        <v>2.13</v>
+        <v>0.69</v>
       </c>
       <c r="AM88">
-        <v>0.16</v>
+        <v>0.03</v>
       </c>
       <c r="AN88">
-        <v>0.12</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="AO88">
-        <v>0.56999999999999995</v>
+        <v>1.49</v>
       </c>
       <c r="AP88">
-        <v>2.25</v>
+        <v>0.75</v>
       </c>
       <c r="AQ88">
-        <v>1.31</v>
+        <v>2.82</v>
       </c>
       <c r="AR88">
-        <v>1.47</v>
+        <v>1.07</v>
       </c>
       <c r="AS88">
-        <v>254</v>
+        <v>667</v>
       </c>
       <c r="AT88">
-        <v>581</v>
+        <v>349</v>
       </c>
       <c r="AU88">
-        <v>73</v>
+        <v>353</v>
       </c>
       <c r="AV88">
-        <v>269</v>
+        <v>129</v>
       </c>
       <c r="AW88">
-        <v>108</v>
+        <v>252</v>
       </c>
       <c r="AX88">
-        <v>252</v>
+        <v>151</v>
       </c>
       <c r="AY88">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="AZ88">
         <v>19</v>
       </c>
       <c r="BA88">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BB88">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BC88">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="BD88">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="BE88">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="BF88">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="BG88">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH88">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BI88" t="s">
         <v>89</v>
@@ -24312,64 +24315,64 @@
         <v>89</v>
       </c>
       <c r="BK88">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="BL88">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="BM88">
         <v>9</v>
       </c>
       <c r="BN88">
+        <v>9</v>
+      </c>
+      <c r="BO88">
+        <v>2</v>
+      </c>
+      <c r="BP88">
+        <v>2</v>
+      </c>
+      <c r="BQ88">
+        <v>17</v>
+      </c>
+      <c r="BR88">
+        <v>15</v>
+      </c>
+      <c r="BS88">
+        <v>4</v>
+      </c>
+      <c r="BT88">
+        <v>3</v>
+      </c>
+      <c r="BU88" t="s">
+        <v>89</v>
+      </c>
+      <c r="BV88" t="s">
+        <v>89</v>
+      </c>
+      <c r="BW88">
+        <v>49</v>
+      </c>
+      <c r="BX88">
+        <v>45</v>
+      </c>
+      <c r="BY88">
+        <v>42</v>
+      </c>
+      <c r="BZ88">
+        <v>39</v>
+      </c>
+      <c r="CA88">
         <v>7</v>
       </c>
-      <c r="BO88">
-        <v>8</v>
-      </c>
-      <c r="BP88">
-        <v>4</v>
-      </c>
-      <c r="BQ88">
-        <v>27</v>
-      </c>
-      <c r="BR88">
-        <v>27</v>
-      </c>
-      <c r="BS88">
-        <v>4</v>
-      </c>
-      <c r="BT88">
-        <v>3</v>
-      </c>
-      <c r="BU88" t="s">
-        <v>89</v>
-      </c>
-      <c r="BV88" t="s">
-        <v>89</v>
-      </c>
-      <c r="BW88">
-        <v>37</v>
-      </c>
-      <c r="BX88">
-        <v>36</v>
-      </c>
-      <c r="BY88">
-        <v>26</v>
-      </c>
-      <c r="BZ88">
-        <v>23</v>
-      </c>
-      <c r="CA88">
+      <c r="CB88">
+        <v>6</v>
+      </c>
+      <c r="CC88">
         <v>11</v>
       </c>
-      <c r="CB88">
-        <v>13</v>
-      </c>
-      <c r="CC88">
-        <v>5</v>
-      </c>
       <c r="CD88">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="CE88" t="s">
         <v>89</v>
@@ -24378,13 +24381,13 @@
         <v>89</v>
       </c>
       <c r="CG88">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="CH88">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CI88">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CJ88">
         <v>0</v>
@@ -24392,13 +24395,13 @@
     </row>
     <row r="89" spans="2:88" ht="30">
       <c r="B89" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="C89" s="4" t="s">
-        <v>87</v>
+        <v>191</v>
+      </c>
+      <c r="C89" t="s">
+        <v>88</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -24407,250 +24410,514 @@
         <v>1</v>
       </c>
       <c r="G89">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="H89">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="I89">
-        <v>1.51</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="J89">
-        <v>0.47</v>
+        <v>2.25</v>
       </c>
       <c r="K89">
+        <v>12</v>
+      </c>
+      <c r="L89">
+        <v>21</v>
+      </c>
+      <c r="M89">
+        <v>4</v>
+      </c>
+      <c r="N89">
+        <v>5</v>
+      </c>
+      <c r="O89">
+        <v>1</v>
+      </c>
+      <c r="P89">
+        <v>3</v>
+      </c>
+      <c r="Q89">
+        <v>0</v>
+      </c>
+      <c r="R89">
+        <v>2</v>
+      </c>
+      <c r="S89">
+        <v>181</v>
+      </c>
+      <c r="T89">
+        <v>521</v>
+      </c>
+      <c r="U89">
+        <v>12</v>
+      </c>
+      <c r="V89">
+        <v>9</v>
+      </c>
+      <c r="W89">
+        <v>8</v>
+      </c>
+      <c r="X89">
+        <v>8</v>
+      </c>
+      <c r="Y89" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z89" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA89">
+        <v>4</v>
+      </c>
+      <c r="AB89">
+        <v>8</v>
+      </c>
+      <c r="AC89">
+        <v>4</v>
+      </c>
+      <c r="AD89">
+        <v>8</v>
+      </c>
+      <c r="AE89">
+        <v>1</v>
+      </c>
+      <c r="AF89">
+        <v>0</v>
+      </c>
+      <c r="AG89">
+        <v>4</v>
+      </c>
+      <c r="AH89">
+        <v>8</v>
+      </c>
+      <c r="AI89">
+        <v>8</v>
+      </c>
+      <c r="AJ89">
+        <v>13</v>
+      </c>
+      <c r="AK89">
+        <v>0.41</v>
+      </c>
+      <c r="AL89">
+        <v>2.13</v>
+      </c>
+      <c r="AM89">
+        <v>0.16</v>
+      </c>
+      <c r="AN89">
+        <v>0.12</v>
+      </c>
+      <c r="AO89">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="AP89">
+        <v>2.25</v>
+      </c>
+      <c r="AQ89">
+        <v>1.31</v>
+      </c>
+      <c r="AR89">
+        <v>1.47</v>
+      </c>
+      <c r="AS89">
+        <v>254</v>
+      </c>
+      <c r="AT89">
+        <v>581</v>
+      </c>
+      <c r="AU89">
+        <v>73</v>
+      </c>
+      <c r="AV89">
+        <v>269</v>
+      </c>
+      <c r="AW89">
+        <v>108</v>
+      </c>
+      <c r="AX89">
+        <v>252</v>
+      </c>
+      <c r="AY89">
+        <v>22</v>
+      </c>
+      <c r="AZ89">
+        <v>19</v>
+      </c>
+      <c r="BA89">
+        <v>5</v>
+      </c>
+      <c r="BB89">
+        <v>4</v>
+      </c>
+      <c r="BC89">
+        <v>13</v>
+      </c>
+      <c r="BD89">
+        <v>15</v>
+      </c>
+      <c r="BE89">
+        <v>10</v>
+      </c>
+      <c r="BF89">
         <v>18</v>
       </c>
-      <c r="L89">
-        <v>7</v>
-      </c>
-      <c r="M89">
-        <v>4</v>
-      </c>
-      <c r="N89">
-        <v>3</v>
-      </c>
-      <c r="O89">
-        <v>1</v>
-      </c>
-      <c r="P89">
-        <v>1</v>
-      </c>
-      <c r="Q89">
-        <v>0</v>
-      </c>
-      <c r="R89">
-        <v>0</v>
-      </c>
-      <c r="S89">
-        <v>367</v>
-      </c>
-      <c r="T89">
-        <v>385</v>
-      </c>
-      <c r="U89">
-        <v>14</v>
-      </c>
-      <c r="V89">
-        <v>12</v>
-      </c>
-      <c r="W89">
-        <v>7</v>
-      </c>
-      <c r="X89">
-        <v>2</v>
-      </c>
-      <c r="Y89" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z89" t="s">
-        <v>89</v>
-      </c>
-      <c r="AA89">
-        <v>8</v>
-      </c>
-      <c r="AB89">
-        <v>4</v>
-      </c>
-      <c r="AC89">
-        <v>6</v>
-      </c>
-      <c r="AD89">
-        <v>0</v>
-      </c>
-      <c r="AE89">
-        <v>2</v>
-      </c>
-      <c r="AF89">
-        <v>0</v>
-      </c>
-      <c r="AG89">
-        <v>12</v>
-      </c>
-      <c r="AH89">
-        <v>5</v>
-      </c>
-      <c r="AI89">
-        <v>6</v>
-      </c>
-      <c r="AJ89">
-        <v>2</v>
-      </c>
-      <c r="AK89">
-        <v>0.81</v>
-      </c>
-      <c r="AL89">
-        <v>0.47</v>
-      </c>
-      <c r="AM89">
-        <v>0.71</v>
-      </c>
-      <c r="AN89">
-        <v>0</v>
-      </c>
-      <c r="AO89">
-        <v>1.51</v>
-      </c>
-      <c r="AP89">
-        <v>0.47</v>
-      </c>
-      <c r="AQ89">
-        <v>1.27</v>
-      </c>
-      <c r="AR89">
-        <v>0.67</v>
-      </c>
-      <c r="AS89">
-        <v>424</v>
-      </c>
-      <c r="AT89">
-        <v>465</v>
-      </c>
-      <c r="AU89">
-        <v>187</v>
-      </c>
-      <c r="AV89">
-        <v>221</v>
-      </c>
-      <c r="AW89">
-        <v>180</v>
-      </c>
-      <c r="AX89">
-        <v>164</v>
-      </c>
-      <c r="AY89">
-        <v>29</v>
-      </c>
-      <c r="AZ89">
-        <v>23</v>
-      </c>
-      <c r="BA89">
+      <c r="BG89">
+        <v>0</v>
+      </c>
+      <c r="BH89">
+        <v>3</v>
+      </c>
+      <c r="BI89" t="s">
+        <v>89</v>
+      </c>
+      <c r="BJ89" t="s">
+        <v>89</v>
+      </c>
+      <c r="BK89">
+        <v>13</v>
+      </c>
+      <c r="BL89">
         <v>10</v>
       </c>
-      <c r="BB89">
-        <v>1</v>
-      </c>
-      <c r="BC89">
-        <v>32</v>
-      </c>
-      <c r="BD89">
-        <v>22</v>
-      </c>
-      <c r="BE89">
-        <v>29</v>
-      </c>
-      <c r="BF89">
-        <v>11</v>
-      </c>
-      <c r="BG89">
-        <v>0</v>
-      </c>
-      <c r="BH89">
-        <v>2</v>
-      </c>
-      <c r="BI89" t="s">
-        <v>89</v>
-      </c>
-      <c r="BJ89" t="s">
-        <v>89</v>
-      </c>
-      <c r="BK89">
-        <v>24</v>
-      </c>
-      <c r="BL89">
-        <v>27</v>
-      </c>
       <c r="BM89">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BN89">
         <v>7</v>
       </c>
       <c r="BO89">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BP89">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BQ89">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="BR89">
+        <v>27</v>
+      </c>
+      <c r="BS89">
+        <v>4</v>
+      </c>
+      <c r="BT89">
+        <v>3</v>
+      </c>
+      <c r="BU89" t="s">
+        <v>89</v>
+      </c>
+      <c r="BV89" t="s">
+        <v>89</v>
+      </c>
+      <c r="BW89">
         <v>37</v>
       </c>
-      <c r="BS89">
-        <v>2</v>
-      </c>
-      <c r="BT89">
-        <v>3</v>
-      </c>
-      <c r="BU89" t="s">
-        <v>89</v>
-      </c>
-      <c r="BV89" t="s">
-        <v>89</v>
-      </c>
-      <c r="BW89">
-        <v>51</v>
-      </c>
       <c r="BX89">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="BY89">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="BZ89">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="CA89">
         <v>11</v>
       </c>
       <c r="CB89">
+        <v>13</v>
+      </c>
+      <c r="CC89">
+        <v>5</v>
+      </c>
+      <c r="CD89">
+        <v>2</v>
+      </c>
+      <c r="CE89" t="s">
+        <v>89</v>
+      </c>
+      <c r="CF89" t="s">
+        <v>89</v>
+      </c>
+      <c r="CG89">
+        <v>6</v>
+      </c>
+      <c r="CH89">
+        <v>3</v>
+      </c>
+      <c r="CI89">
+        <v>1</v>
+      </c>
+      <c r="CJ89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="2:88" ht="30">
+      <c r="B90" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+      <c r="G90">
+        <v>50</v>
+      </c>
+      <c r="H90">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="I90">
+        <v>1.51</v>
+      </c>
+      <c r="J90">
+        <v>0.47</v>
+      </c>
+      <c r="K90">
+        <v>18</v>
+      </c>
+      <c r="L90">
+        <v>7</v>
+      </c>
+      <c r="M90">
+        <v>4</v>
+      </c>
+      <c r="N90">
+        <v>3</v>
+      </c>
+      <c r="O90">
+        <v>1</v>
+      </c>
+      <c r="P90">
+        <v>1</v>
+      </c>
+      <c r="Q90">
+        <v>0</v>
+      </c>
+      <c r="R90">
+        <v>0</v>
+      </c>
+      <c r="S90">
+        <v>367</v>
+      </c>
+      <c r="T90">
+        <v>385</v>
+      </c>
+      <c r="U90">
+        <v>14</v>
+      </c>
+      <c r="V90">
+        <v>12</v>
+      </c>
+      <c r="W90">
+        <v>7</v>
+      </c>
+      <c r="X90">
+        <v>2</v>
+      </c>
+      <c r="Y90" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z90" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA90">
+        <v>8</v>
+      </c>
+      <c r="AB90">
+        <v>4</v>
+      </c>
+      <c r="AC90">
+        <v>6</v>
+      </c>
+      <c r="AD90">
+        <v>0</v>
+      </c>
+      <c r="AE90">
+        <v>2</v>
+      </c>
+      <c r="AF90">
+        <v>0</v>
+      </c>
+      <c r="AG90">
+        <v>12</v>
+      </c>
+      <c r="AH90">
+        <v>5</v>
+      </c>
+      <c r="AI90">
+        <v>6</v>
+      </c>
+      <c r="AJ90">
+        <v>2</v>
+      </c>
+      <c r="AK90">
+        <v>0.81</v>
+      </c>
+      <c r="AL90">
+        <v>0.47</v>
+      </c>
+      <c r="AM90">
+        <v>0.71</v>
+      </c>
+      <c r="AN90">
+        <v>0</v>
+      </c>
+      <c r="AO90">
+        <v>1.51</v>
+      </c>
+      <c r="AP90">
+        <v>0.47</v>
+      </c>
+      <c r="AQ90">
+        <v>1.27</v>
+      </c>
+      <c r="AR90">
+        <v>0.67</v>
+      </c>
+      <c r="AS90">
+        <v>424</v>
+      </c>
+      <c r="AT90">
+        <v>465</v>
+      </c>
+      <c r="AU90">
+        <v>187</v>
+      </c>
+      <c r="AV90">
+        <v>221</v>
+      </c>
+      <c r="AW90">
+        <v>180</v>
+      </c>
+      <c r="AX90">
+        <v>164</v>
+      </c>
+      <c r="AY90">
+        <v>29</v>
+      </c>
+      <c r="AZ90">
+        <v>23</v>
+      </c>
+      <c r="BA90">
+        <v>10</v>
+      </c>
+      <c r="BB90">
+        <v>1</v>
+      </c>
+      <c r="BC90">
+        <v>32</v>
+      </c>
+      <c r="BD90">
+        <v>22</v>
+      </c>
+      <c r="BE90">
+        <v>29</v>
+      </c>
+      <c r="BF90">
+        <v>11</v>
+      </c>
+      <c r="BG90">
+        <v>0</v>
+      </c>
+      <c r="BH90">
+        <v>2</v>
+      </c>
+      <c r="BI90" t="s">
+        <v>89</v>
+      </c>
+      <c r="BJ90" t="s">
+        <v>89</v>
+      </c>
+      <c r="BK90">
+        <v>24</v>
+      </c>
+      <c r="BL90">
+        <v>27</v>
+      </c>
+      <c r="BM90">
+        <v>8</v>
+      </c>
+      <c r="BN90">
+        <v>7</v>
+      </c>
+      <c r="BO90">
+        <v>0</v>
+      </c>
+      <c r="BP90">
+        <v>6</v>
+      </c>
+      <c r="BQ90">
         <v>16</v>
       </c>
-      <c r="CC89">
-        <v>5</v>
-      </c>
-      <c r="CD89">
+      <c r="BR90">
+        <v>37</v>
+      </c>
+      <c r="BS90">
+        <v>2</v>
+      </c>
+      <c r="BT90">
+        <v>3</v>
+      </c>
+      <c r="BU90" t="s">
+        <v>89</v>
+      </c>
+      <c r="BV90" t="s">
+        <v>89</v>
+      </c>
+      <c r="BW90">
+        <v>51</v>
+      </c>
+      <c r="BX90">
+        <v>63</v>
+      </c>
+      <c r="BY90">
+        <v>40</v>
+      </c>
+      <c r="BZ90">
+        <v>47</v>
+      </c>
+      <c r="CA90">
+        <v>11</v>
+      </c>
+      <c r="CB90">
+        <v>16</v>
+      </c>
+      <c r="CC90">
+        <v>5</v>
+      </c>
+      <c r="CD90">
         <v>6</v>
       </c>
-      <c r="CE89" t="s">
-        <v>89</v>
-      </c>
-      <c r="CF89" t="s">
-        <v>89</v>
-      </c>
-      <c r="CG89">
-        <v>2</v>
-      </c>
-      <c r="CH89">
-        <v>1</v>
-      </c>
-      <c r="CI89">
-        <v>0</v>
-      </c>
-      <c r="CJ89">
+      <c r="CE90" t="s">
+        <v>89</v>
+      </c>
+      <c r="CF90" t="s">
+        <v>89</v>
+      </c>
+      <c r="CG90">
+        <v>2</v>
+      </c>
+      <c r="CH90">
+        <v>1</v>
+      </c>
+      <c r="CI90">
+        <v>0</v>
+      </c>
+      <c r="CJ90">
         <v>0</v>
       </c>
     </row>

</xml_diff>